<commit_message>
C12 · Recibidas con las columnas de Julio; fuera la prueba de la URL corta (Julio: enlace permanente con llave)
- El Excel de prueba de recibidas sigue la configuración de Julio
  (ConfiguracionRecibidas.XML) tal cual, con «Url documento» en la K (Campo056,
  el que funcionó en emitidas) y la retención en T/U/V, a mano.
- Julio decide el enlace permanente con llave por documento: se quitan los dos
  trabajos de la URL corta y su script.
- traspaso-completo.md: las decisiones de Julio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012QT7a1DXYVhNd7XC8w2p8z
</commit_message>
<xml_diff>
--- a/docs/conta/c12/prueba-excel/prueba-c12-recibidas-url.xlsx
+++ b/docs/conta/c12/prueba-excel/prueba-c12-recibidas-url.xlsx
@@ -399,130 +399,127 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:V4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Nº factura</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Fecha</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Fecha</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Nombre</v>
+      </c>
+      <c r="E1" t="str">
+        <v>% IVA 1</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Cuota IVA 1</v>
+      </c>
+      <c r="G1" t="str">
         <v>Subcuenta proveedor</v>
       </c>
-      <c r="B1" t="str">
+      <c r="H1" t="str">
         <v>Concepto asiento</v>
       </c>
-      <c r="C1" t="str">
-        <v>Nombre</v>
-      </c>
-      <c r="D1" t="str">
-        <v>NIF</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Subcuenta gasto 1</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Nº factura</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Importe gasto 1</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Subcuenta gasto 2</v>
-      </c>
       <c r="I1" t="str">
-        <v>Importe gasto 2</v>
+        <v>Base IVA 1</v>
       </c>
       <c r="J1" t="str">
-        <v/>
+        <v>Total factura</v>
       </c>
       <c r="K1" t="str">
         <v>Url documento</v>
       </c>
       <c r="L1" t="str">
-        <v/>
+        <v>Subcuenta gasto 1</v>
       </c>
       <c r="M1" t="str">
-        <v>Base IVA 1</v>
+        <v>Importe gasto 1</v>
       </c>
       <c r="N1" t="str">
-        <v>% IVA 1</v>
+        <v>Ruta documento</v>
       </c>
       <c r="O1" t="str">
-        <v>Cuota IVA 1</v>
+        <v>Base IVA 2</v>
       </c>
       <c r="P1" t="str">
-        <v>Total factura</v>
+        <v>% IVA 2</v>
       </c>
       <c r="Q1" t="str">
-        <v>Fecha</v>
+        <v>Cuota IVA 2</v>
       </c>
       <c r="R1" t="str">
-        <v>Base IVA 2</v>
+        <v>Subcuenta gasto 2</v>
       </c>
       <c r="S1" t="str">
-        <v>% IVA 2</v>
+        <v>Importe gasto 2</v>
       </c>
       <c r="T1" t="str">
-        <v>Cuota IVA 2</v>
+        <v>Base retención</v>
       </c>
       <c r="U1" t="str">
-        <v>Base retención</v>
+        <v>% retención</v>
       </c>
       <c r="V1" t="str">
-        <v>% retención</v>
-      </c>
-      <c r="W1" t="str">
         <v>Cuota retención</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>PRB-C12-R001</v>
+      </c>
+      <c r="B2" s="1" t="d">
+        <v>2026-10-24T00:00:00.000Z</v>
+      </c>
+      <c r="C2" s="1" t="d">
+        <v>2026-10-24T00:00:00.000Z</v>
+      </c>
+      <c r="D2" t="str">
+        <v>PROVEEDOR PRUEBA C12</v>
+      </c>
+      <c r="E2">
+        <v>21</v>
+      </c>
+      <c r="F2">
+        <v>21</v>
+      </c>
+      <c r="G2" t="str">
         <v>40000990</v>
       </c>
-      <c r="B2" t="str">
+      <c r="H2" t="str">
         <v>Prueba C12 · recibida normal</v>
       </c>
-      <c r="C2" t="str">
-        <v>PROVEEDOR PRUEBA C12</v>
-      </c>
-      <c r="D2" t="str">
-        <v>B00000001</v>
-      </c>
-      <c r="E2" t="str">
-        <v>60000000</v>
-      </c>
-      <c r="F2" t="str">
-        <v>PRB-C12-R001</v>
-      </c>
-      <c r="G2">
+      <c r="I2">
         <v>100</v>
       </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
+      <c r="J2">
+        <v>121</v>
       </c>
       <c r="K2" t="str">
         <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>60000000</v>
       </c>
       <c r="M2">
         <v>100</v>
       </c>
-      <c r="N2">
-        <v>21</v>
-      </c>
-      <c r="O2">
-        <v>21</v>
-      </c>
-      <c r="P2">
-        <v>121</v>
-      </c>
-      <c r="Q2" s="1" t="d">
-        <v>2026-10-24T00:00:00.000Z</v>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
       </c>
       <c r="R2" t="str">
         <v/>
@@ -537,134 +534,128 @@
         <v/>
       </c>
       <c r="V2" t="str">
-        <v/>
-      </c>
-      <c r="W2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>PRB-C12-R002</v>
+      </c>
+      <c r="B3" s="1" t="d">
+        <v>2026-10-24T00:00:00.000Z</v>
+      </c>
+      <c r="C3" s="1" t="d">
+        <v>2026-10-24T00:00:00.000Z</v>
+      </c>
+      <c r="D3" t="str">
+        <v>PROVEEDOR PRUEBA C12</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+      <c r="G3" t="str">
         <v>40000990</v>
       </c>
-      <c r="B3" t="str">
+      <c r="H3" t="str">
         <v>Prueba C12 · recibida con dos tipos de IVA</v>
       </c>
-      <c r="C3" t="str">
-        <v>PROVEEDOR PRUEBA C12</v>
-      </c>
-      <c r="D3" t="str">
-        <v>B00000001</v>
-      </c>
-      <c r="E3" t="str">
-        <v>60000000</v>
-      </c>
-      <c r="F3" t="str">
-        <v>PRB-C12-R002</v>
-      </c>
-      <c r="G3">
+      <c r="I3">
         <v>100</v>
       </c>
-      <c r="H3" t="str">
-        <v>62900000</v>
-      </c>
-      <c r="I3">
-        <v>50</v>
-      </c>
-      <c r="J3" t="str">
-        <v/>
+      <c r="J3">
+        <v>170.5</v>
       </c>
       <c r="K3" t="str">
         <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>60000000</v>
       </c>
       <c r="M3">
         <v>100</v>
       </c>
-      <c r="N3">
-        <v>10</v>
+      <c r="N3" t="str">
+        <v/>
       </c>
       <c r="O3">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="P3">
-        <v>170.5</v>
-      </c>
-      <c r="Q3" s="1" t="d">
-        <v>2026-10-24T00:00:00.000Z</v>
-      </c>
-      <c r="R3">
+        <v>21</v>
+      </c>
+      <c r="Q3">
+        <v>10.5</v>
+      </c>
+      <c r="R3" t="str">
+        <v>62900000</v>
+      </c>
+      <c r="S3">
         <v>50</v>
       </c>
-      <c r="S3">
-        <v>21</v>
-      </c>
-      <c r="T3">
-        <v>10.5</v>
+      <c r="T3" t="str">
+        <v/>
       </c>
       <c r="U3" t="str">
         <v/>
       </c>
       <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>PRB-C12-R003</v>
+      </c>
+      <c r="B4" s="1" t="d">
+        <v>2026-10-24T00:00:00.000Z</v>
+      </c>
+      <c r="C4" s="1" t="d">
+        <v>2026-10-24T00:00:00.000Z</v>
+      </c>
+      <c r="D4" t="str">
+        <v>PROVEEDOR PRUEBA C12</v>
+      </c>
+      <c r="E4">
+        <v>21</v>
+      </c>
+      <c r="F4">
+        <v>42</v>
+      </c>
+      <c r="G4" t="str">
         <v>40000990</v>
       </c>
-      <c r="B4" t="str">
+      <c r="H4" t="str">
         <v>Prueba C12 · profesional con retención</v>
       </c>
-      <c r="C4" t="str">
-        <v>PROVEEDOR PRUEBA C12</v>
-      </c>
-      <c r="D4" t="str">
-        <v>B00000001</v>
-      </c>
-      <c r="E4" t="str">
-        <v>62300000</v>
-      </c>
-      <c r="F4" t="str">
-        <v>PRB-C12-R003</v>
-      </c>
-      <c r="G4">
+      <c r="I4">
         <v>200</v>
       </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
+      <c r="J4">
+        <v>212</v>
       </c>
       <c r="K4" t="str">
         <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>62300000</v>
       </c>
       <c r="M4">
         <v>200</v>
       </c>
-      <c r="N4">
-        <v>21</v>
-      </c>
-      <c r="O4">
-        <v>42</v>
-      </c>
-      <c r="P4">
-        <v>212</v>
-      </c>
-      <c r="Q4" s="1" t="d">
-        <v>2026-10-24T00:00:00.000Z</v>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
       </c>
       <c r="R4" t="str">
         <v/>
@@ -672,22 +663,19 @@
       <c r="S4" t="str">
         <v/>
       </c>
-      <c r="T4" t="str">
-        <v/>
+      <c r="T4">
+        <v>200</v>
       </c>
       <c r="U4">
-        <v>200</v>
+        <v>15</v>
       </c>
       <c r="V4">
-        <v>15</v>
-      </c>
-      <c r="W4">
         <v>30</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
C12 · Recibidas de prueba, segunda: cada dato a la columna del XML de Julio
- La C es el N.I.F. (Campo003), no una fecha: salía «24102026».
- Retención en T/U/V con su tipo PRO en la W (Campo034–037): la R003 entró
  sin ella y el asiento descuadraba en 30 €.
- Las columnas se leen del XML de Julio, que va tal cual; el generador
  vuelve a leer el Excel por ellas y para si algún asiento no cuadra.
- Prueba unitaria contra el XML real y contra los dos fallos de la primera.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012QT7a1DXYVhNd7XC8w2p8z
</commit_message>
<xml_diff>
--- a/docs/conta/c12/prueba-excel/prueba-c12-recibidas-url.xlsx
+++ b/docs/conta/c12/prueba-excel/prueba-c12-recibidas-url.xlsx
@@ -399,17 +399,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:W4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Nº factura</v>
       </c>
       <c r="B1" t="str">
-        <v>Fecha</v>
+        <v>Fecha expedición / Fecha operación</v>
       </c>
       <c r="C1" t="str">
-        <v>Fecha</v>
+        <v>N.I.F.</v>
       </c>
       <c r="D1" t="str">
         <v>Nombre</v>
@@ -467,6 +467,9 @@
       </c>
       <c r="V1" t="str">
         <v>Cuota retención</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Tipo retención</v>
       </c>
     </row>
     <row r="2">
@@ -476,8 +479,8 @@
       <c r="B2" s="1" t="d">
         <v>2026-10-24T00:00:00.000Z</v>
       </c>
-      <c r="C2" s="1" t="d">
-        <v>2026-10-24T00:00:00.000Z</v>
+      <c r="C2" t="str">
+        <v>B00000001</v>
       </c>
       <c r="D2" t="str">
         <v>PROVEEDOR PRUEBA C12</v>
@@ -534,6 +537,9 @@
         <v/>
       </c>
       <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
         <v/>
       </c>
     </row>
@@ -544,8 +550,8 @@
       <c r="B3" s="1" t="d">
         <v>2026-10-24T00:00:00.000Z</v>
       </c>
-      <c r="C3" s="1" t="d">
-        <v>2026-10-24T00:00:00.000Z</v>
+      <c r="C3" t="str">
+        <v>B00000001</v>
       </c>
       <c r="D3" t="str">
         <v>PROVEEDOR PRUEBA C12</v>
@@ -602,6 +608,9 @@
         <v/>
       </c>
       <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
         <v/>
       </c>
     </row>
@@ -612,8 +621,8 @@
       <c r="B4" s="1" t="d">
         <v>2026-10-24T00:00:00.000Z</v>
       </c>
-      <c r="C4" s="1" t="d">
-        <v>2026-10-24T00:00:00.000Z</v>
+      <c r="C4" t="str">
+        <v>B00000001</v>
       </c>
       <c r="D4" t="str">
         <v>PROVEEDOR PRUEBA C12</v>
@@ -671,11 +680,14 @@
       </c>
       <c r="V4">
         <v>30</v>
+      </c>
+      <c r="W4" t="str">
+        <v>PRO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
C12 · Excel de Diez sin fila de títulos; retención con su subcuenta en la X
- Emitidas y recibidas sin fila de títulos: Diez la leía como una factura.
- Recibidas: la subcuenta de la retención en la X (Campo038, XML de Julio),
  la que Sumied enlaza a ese tipo (Profesionales → 47510015, medida en
  Foodint); el generador para si un tipo no la tiene.
- El generador para también si una línea del asiento va sin cuenta o si
  una fila no es una factura.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012QT7a1DXYVhNd7XC8w2p8z
</commit_message>
<xml_diff>
--- a/docs/conta/c12/prueba-excel/prueba-c12-recibidas-url.xlsx
+++ b/docs/conta/c12/prueba-excel/prueba-c12-recibidas-url.xlsx
@@ -399,82 +399,85 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:X3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Nº factura</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Fecha expedición / Fecha operación</v>
+        <v>PRB-C12-R001</v>
+      </c>
+      <c r="B1" s="1" t="d">
+        <v>2026-10-24T00:00:00.000Z</v>
       </c>
       <c r="C1" t="str">
-        <v>N.I.F.</v>
+        <v>B00000001</v>
       </c>
       <c r="D1" t="str">
-        <v>Nombre</v>
-      </c>
-      <c r="E1" t="str">
-        <v>% IVA 1</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Cuota IVA 1</v>
+        <v>PROVEEDOR PRUEBA C12</v>
+      </c>
+      <c r="E1">
+        <v>21</v>
+      </c>
+      <c r="F1">
+        <v>21</v>
       </c>
       <c r="G1" t="str">
-        <v>Subcuenta proveedor</v>
+        <v>40000990</v>
       </c>
       <c r="H1" t="str">
-        <v>Concepto asiento</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Base IVA 1</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Total factura</v>
+        <v>Prueba C12 · recibida normal</v>
+      </c>
+      <c r="I1">
+        <v>100</v>
+      </c>
+      <c r="J1">
+        <v>121</v>
       </c>
       <c r="K1" t="str">
-        <v>Url documento</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
       <c r="L1" t="str">
-        <v>Subcuenta gasto 1</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Importe gasto 1</v>
+        <v>60000000</v>
+      </c>
+      <c r="M1">
+        <v>100</v>
       </c>
       <c r="N1" t="str">
-        <v>Ruta documento</v>
+        <v/>
       </c>
       <c r="O1" t="str">
-        <v>Base IVA 2</v>
+        <v/>
       </c>
       <c r="P1" t="str">
-        <v>% IVA 2</v>
+        <v/>
       </c>
       <c r="Q1" t="str">
-        <v>Cuota IVA 2</v>
+        <v/>
       </c>
       <c r="R1" t="str">
-        <v>Subcuenta gasto 2</v>
+        <v/>
       </c>
       <c r="S1" t="str">
-        <v>Importe gasto 2</v>
+        <v/>
       </c>
       <c r="T1" t="str">
-        <v>Base retención</v>
+        <v/>
       </c>
       <c r="U1" t="str">
-        <v>% retención</v>
+        <v/>
       </c>
       <c r="V1" t="str">
-        <v>Cuota retención</v>
+        <v/>
       </c>
       <c r="W1" t="str">
-        <v>Tipo retención</v>
+        <v/>
+      </c>
+      <c r="X1" t="str">
+        <v/>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>PRB-C12-R001</v>
+        <v>PRB-C12-R002</v>
       </c>
       <c r="B2" s="1" t="d">
         <v>2026-10-24T00:00:00.000Z</v>
@@ -486,22 +489,22 @@
         <v>PROVEEDOR PRUEBA C12</v>
       </c>
       <c r="E2">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F2">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G2" t="str">
         <v>40000990</v>
       </c>
       <c r="H2" t="str">
-        <v>Prueba C12 · recibida normal</v>
+        <v>Prueba C12 · recibida con dos tipos de IVA</v>
       </c>
       <c r="I2">
         <v>100</v>
       </c>
       <c r="J2">
-        <v>121</v>
+        <v>170.5</v>
       </c>
       <c r="K2" t="str">
         <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
@@ -515,20 +518,20 @@
       <c r="N2" t="str">
         <v/>
       </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
+      <c r="O2">
+        <v>50</v>
+      </c>
+      <c r="P2">
+        <v>21</v>
+      </c>
+      <c r="Q2">
+        <v>10.5</v>
       </c>
       <c r="R2" t="str">
-        <v/>
-      </c>
-      <c r="S2" t="str">
-        <v/>
+        <v>62900000</v>
+      </c>
+      <c r="S2">
+        <v>50</v>
       </c>
       <c r="T2" t="str">
         <v/>
@@ -540,12 +543,15 @@
         <v/>
       </c>
       <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>PRB-C12-R002</v>
+        <v>PRB-C12-R003</v>
       </c>
       <c r="B3" s="1" t="d">
         <v>2026-10-24T00:00:00.000Z</v>
@@ -557,137 +563,69 @@
         <v>PROVEEDOR PRUEBA C12</v>
       </c>
       <c r="E3">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F3">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="G3" t="str">
         <v>40000990</v>
       </c>
       <c r="H3" t="str">
-        <v>Prueba C12 · recibida con dos tipos de IVA</v>
+        <v>Prueba C12 · profesional con retención</v>
       </c>
       <c r="I3">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J3">
-        <v>170.5</v>
+        <v>212</v>
       </c>
       <c r="K3" t="str">
         <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
       <c r="L3" t="str">
-        <v>60000000</v>
+        <v>62300000</v>
       </c>
       <c r="M3">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="N3" t="str">
         <v/>
       </c>
-      <c r="O3">
-        <v>50</v>
-      </c>
-      <c r="P3">
-        <v>21</v>
-      </c>
-      <c r="Q3">
-        <v>10.5</v>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
       </c>
       <c r="R3" t="str">
-        <v>62900000</v>
-      </c>
-      <c r="S3">
-        <v>50</v>
-      </c>
-      <c r="T3" t="str">
-        <v/>
-      </c>
-      <c r="U3" t="str">
-        <v/>
-      </c>
-      <c r="V3" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3">
+        <v>200</v>
+      </c>
+      <c r="U3">
+        <v>15</v>
+      </c>
+      <c r="V3">
+        <v>30</v>
       </c>
       <c r="W3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>PRB-C12-R003</v>
-      </c>
-      <c r="B4" s="1" t="d">
-        <v>2026-10-24T00:00:00.000Z</v>
-      </c>
-      <c r="C4" t="str">
-        <v>B00000001</v>
-      </c>
-      <c r="D4" t="str">
-        <v>PROVEEDOR PRUEBA C12</v>
-      </c>
-      <c r="E4">
-        <v>21</v>
-      </c>
-      <c r="F4">
-        <v>42</v>
-      </c>
-      <c r="G4" t="str">
-        <v>40000990</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Prueba C12 · profesional con retención</v>
-      </c>
-      <c r="I4">
-        <v>200</v>
-      </c>
-      <c r="J4">
-        <v>212</v>
-      </c>
-      <c r="K4" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
-      </c>
-      <c r="L4" t="str">
-        <v>62300000</v>
-      </c>
-      <c r="M4">
-        <v>200</v>
-      </c>
-      <c r="N4" t="str">
-        <v/>
-      </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4" t="str">
-        <v/>
-      </c>
-      <c r="S4" t="str">
-        <v/>
-      </c>
-      <c r="T4">
-        <v>200</v>
-      </c>
-      <c r="U4">
-        <v>15</v>
-      </c>
-      <c r="V4">
-        <v>30</v>
-      </c>
-      <c r="W4" t="str">
         <v>PRO</v>
+      </c>
+      <c r="X3" t="str">
+        <v>47510015</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>